<commit_message>
chore: version final 30Set
</commit_message>
<xml_diff>
--- a/factoring_project/factoring_web/public/plantilla/plantilla_ejemplo.xlsx
+++ b/factoring_project/factoring_web/public/plantilla/plantilla_ejemplo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Apps\CursoArqTecsup\github\tecsup-arq-factoring-dist\factoring_project\factoring_web\public\plantilla\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8B62692F-7143-4E90-AAB2-111E07B0E185}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B33DE8E0-7C96-4054-A6D0-D7CC0EE14E4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11235" xr2:uid="{CAEB4648-BE6A-415B-8428-A90F76E7F78F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{CAEB4648-BE6A-415B-8428-A90F76E7F78F}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -573,7 +573,9 @@
     <col min="8" max="8" width="10.85546875" style="7" customWidth="1"/>
     <col min="9" max="9" width="18.42578125" style="7" customWidth="1"/>
     <col min="10" max="10" width="18.7109375" style="7" customWidth="1"/>
-    <col min="11" max="16384" width="11.42578125" style="7"/>
+    <col min="11" max="14" width="11.42578125" style="7"/>
+    <col min="15" max="15" width="21.28515625" style="7" customWidth="1"/>
+    <col min="16" max="16384" width="11.42578125" style="7"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">

</xml_diff>